<commit_message>
update activity cat domain table
</commit_message>
<xml_diff>
--- a/Domain_Tables_20231004.xlsx
+++ b/Domain_Tables_20231004.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1081" uniqueCount="667">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1081" uniqueCount="666">
   <si>
     <t>Field</t>
   </si>
@@ -1265,9 +1265,6 @@
   </si>
   <si>
     <t>Chipping, Dozer, Handline, Landing Treated - Area Mitigated, Lop and Scatter, Mastication/Chaining/Crushing, Mowing, Piling, Precommercial Thinning (Manual), Precommercial Thinning (Mechanical), Pruning, Tree Release and Weed, Trees Felled (&gt; 6in dbh), Yarding/Biomass Removal, Herbicide Application (IF Primary Objective = Fire Prevention, Other Fuels Reduction, Recreation, Roadway Clearance, Utility Right of Way Clearance)</t>
-  </si>
-  <si>
-    <t>BENEFICIAL_FIRE</t>
   </si>
   <si>
     <t>Broadcast Burn, Wildfire Managed for Resource Benefit, Pile Burning</t>
@@ -2036,7 +2033,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="12">
+  <fonts count="11">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -2090,11 +2087,6 @@
     <font>
       <color theme="1"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -2199,7 +2191,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="38">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -2232,6 +2224,9 @@
     </xf>
     <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
@@ -2271,7 +2266,7 @@
     <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -2280,12 +2275,6 @@
     </xf>
     <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -2302,7 +2291,7 @@
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="1" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -4123,85 +4112,85 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>492</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>493</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="D2" s="4" t="s">
         <v>494</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>495</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>496</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
+        <v>496</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>492</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>497</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>493</v>
-      </c>
-      <c r="C3" s="5" t="s">
+      <c r="D3" s="4" t="s">
         <v>498</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>499</v>
       </c>
       <c r="E3" s="4"/>
     </row>
     <row r="4">
       <c r="A4" s="4"/>
       <c r="B4" s="4" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="C4" s="5" t="s">
+        <v>499</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>500</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>501</v>
       </c>
       <c r="E4" s="4"/>
     </row>
     <row r="5">
       <c r="A5" s="4"/>
       <c r="B5" s="4" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="C5" s="5" t="s">
+        <v>501</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>502</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>503</v>
       </c>
       <c r="E5" s="4"/>
     </row>
     <row r="6">
       <c r="A6" s="4"/>
       <c r="B6" s="4" t="s">
-        <v>493</v>
-      </c>
-      <c r="C6" s="15" t="s">
+        <v>492</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>480</v>
+      </c>
+      <c r="D6" s="17" t="s">
         <v>481</v>
-      </c>
-      <c r="D6" s="16" t="s">
-        <v>482</v>
       </c>
       <c r="E6" s="4"/>
     </row>
     <row r="7">
       <c r="A7" s="4"/>
       <c r="B7" s="4" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="C7" s="5" t="s">
+        <v>503</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>504</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>505</v>
       </c>
       <c r="E7" s="4"/>
     </row>
@@ -5227,63 +5216,63 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
+        <v>505</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>506</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="16" t="s">
         <v>507</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="D2" s="17" t="s">
         <v>508</v>
-      </c>
-      <c r="D2" s="16" t="s">
-        <v>509</v>
       </c>
       <c r="E2" s="4"/>
     </row>
     <row r="3">
       <c r="A3" s="4"/>
       <c r="B3" s="4" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="C3" s="5" t="s">
+        <v>509</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>510</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>511</v>
       </c>
       <c r="E3" s="4"/>
     </row>
     <row r="4">
       <c r="A4" s="4"/>
       <c r="B4" s="4" t="s">
-        <v>507</v>
-      </c>
-      <c r="C4" s="15" t="s">
+        <v>506</v>
+      </c>
+      <c r="C4" s="16" t="s">
+        <v>511</v>
+      </c>
+      <c r="D4" s="17" t="s">
         <v>512</v>
-      </c>
-      <c r="D4" s="16" t="s">
-        <v>513</v>
       </c>
       <c r="E4" s="4"/>
     </row>
     <row r="5">
       <c r="A5" s="4"/>
       <c r="B5" s="4" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="C5" s="5" t="s">
+        <v>513</v>
+      </c>
+      <c r="D5" s="17" t="s">
         <v>514</v>
       </c>
-      <c r="D5" s="16" t="s">
-        <v>515</v>
-      </c>
       <c r="E5" s="4"/>
     </row>
     <row r="6">
-      <c r="C6" s="14" t="s">
+      <c r="C6" s="15" t="s">
         <v>230</v>
       </c>
-      <c r="D6" s="17" t="s">
+      <c r="D6" s="18" t="s">
         <v>231</v>
       </c>
     </row>
@@ -6309,94 +6298,94 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
+        <v>515</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>516</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>517</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="D2" s="17" t="s">
         <v>518</v>
-      </c>
-      <c r="D2" s="16" t="s">
-        <v>519</v>
       </c>
       <c r="E2" s="4"/>
     </row>
     <row r="3">
       <c r="A3" s="4"/>
       <c r="B3" s="4" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="C3" s="5" t="s">
+        <v>519</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>520</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>521</v>
       </c>
       <c r="E3" s="4"/>
     </row>
     <row r="4">
       <c r="A4" s="4"/>
       <c r="B4" s="4" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="E4" s="4"/>
     </row>
     <row r="5">
       <c r="A5" s="4"/>
       <c r="B5" s="4" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="C5" s="5" t="s">
+        <v>522</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>523</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>524</v>
       </c>
       <c r="E5" s="4"/>
     </row>
     <row r="6">
       <c r="A6" s="4"/>
       <c r="B6" s="4" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="C6" s="5" t="s">
+        <v>524</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>525</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>526</v>
       </c>
       <c r="E6" s="4"/>
     </row>
     <row r="7">
       <c r="A7" s="4"/>
       <c r="B7" s="4" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="C7" s="5" t="s">
+        <v>526</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>527</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>528</v>
       </c>
       <c r="E7" s="4"/>
     </row>
     <row r="8">
       <c r="A8" s="4"/>
       <c r="B8" s="4" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="C8" s="5" t="s">
+        <v>528</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>529</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>530</v>
       </c>
       <c r="E8" s="4"/>
     </row>
@@ -7421,144 +7410,144 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="19" t="s">
+        <v>530</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>531</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="4" t="s">
         <v>532</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="D2" s="13" t="s">
         <v>533</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="E2" s="4"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="19" t="s">
         <v>534</v>
       </c>
-      <c r="E2" s="4"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="18" t="s">
+      <c r="B3" s="4" t="s">
+        <v>531</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>535</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>532</v>
-      </c>
-      <c r="C3" s="4" t="s">
+      <c r="D3" s="13" t="s">
         <v>536</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="E3" s="4"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="19" t="s">
         <v>537</v>
       </c>
-      <c r="E3" s="4"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="18" t="s">
+      <c r="B4" s="4" t="s">
+        <v>531</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>538</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>532</v>
-      </c>
-      <c r="C4" s="4" t="s">
+      <c r="D4" s="13" t="s">
         <v>539</v>
-      </c>
-      <c r="D4" s="12" t="s">
-        <v>540</v>
       </c>
       <c r="E4" s="4"/>
     </row>
     <row r="5">
       <c r="A5" s="4"/>
       <c r="B5" s="4" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="C5" s="4" t="s">
+        <v>540</v>
+      </c>
+      <c r="D5" s="13" t="s">
         <v>541</v>
-      </c>
-      <c r="D5" s="12" t="s">
-        <v>542</v>
       </c>
       <c r="E5" s="4"/>
     </row>
     <row r="6">
       <c r="A6" s="4"/>
       <c r="B6" s="4" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="C6" s="4" t="s">
+        <v>542</v>
+      </c>
+      <c r="D6" s="13" t="s">
         <v>543</v>
-      </c>
-      <c r="D6" s="12" t="s">
-        <v>544</v>
       </c>
       <c r="E6" s="4"/>
     </row>
     <row r="7">
       <c r="A7" s="4"/>
       <c r="B7" s="4" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="C7" s="4" t="s">
+        <v>544</v>
+      </c>
+      <c r="D7" s="13" t="s">
         <v>545</v>
-      </c>
-      <c r="D7" s="12" t="s">
-        <v>546</v>
       </c>
       <c r="E7" s="4"/>
     </row>
     <row r="8">
       <c r="A8" s="4"/>
       <c r="B8" s="4" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="C8" s="4" t="s">
+        <v>546</v>
+      </c>
+      <c r="D8" s="13" t="s">
         <v>547</v>
-      </c>
-      <c r="D8" s="12" t="s">
-        <v>548</v>
       </c>
       <c r="E8" s="4"/>
     </row>
     <row r="9">
       <c r="B9" s="4" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="C9" s="4" t="s">
+        <v>548</v>
+      </c>
+      <c r="D9" s="13" t="s">
         <v>549</v>
-      </c>
-      <c r="D9" s="12" t="s">
-        <v>550</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="4" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="C10" s="4" t="s">
+        <v>517</v>
+      </c>
+      <c r="D10" s="13" t="s">
         <v>518</v>
-      </c>
-      <c r="D10" s="12" t="s">
-        <v>519</v>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="4" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="C11" s="4" t="s">
+        <v>519</v>
+      </c>
+      <c r="D11" s="13" t="s">
         <v>520</v>
-      </c>
-      <c r="D11" s="12" t="s">
-        <v>521</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="4" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="C12" s="4" t="s">
+        <v>550</v>
+      </c>
+      <c r="D12" s="13" t="s">
         <v>551</v>
-      </c>
-      <c r="D12" s="12" t="s">
-        <v>552</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -8565,157 +8554,157 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20" t="s">
+      <c r="B1" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="21" t="s">
+      <c r="C1" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="20" t="s">
+      <c r="D1" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="22" t="s">
+      <c r="E1" s="23" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="24" t="s">
+        <v>552</v>
+      </c>
+      <c r="B2" s="25" t="s">
         <v>553</v>
       </c>
-      <c r="B2" s="24" t="s">
+      <c r="C2" s="24" t="s">
         <v>554</v>
       </c>
-      <c r="C2" s="23" t="s">
+      <c r="D2" s="25" t="s">
         <v>555</v>
       </c>
-      <c r="D2" s="24" t="s">
+      <c r="E2" s="26"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="25"/>
+      <c r="B3" s="25" t="s">
+        <v>553</v>
+      </c>
+      <c r="C3" s="24" t="s">
         <v>556</v>
       </c>
-      <c r="E2" s="25"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="24"/>
-      <c r="B3" s="24" t="s">
-        <v>554</v>
-      </c>
-      <c r="C3" s="23" t="s">
+      <c r="D3" s="25" t="s">
         <v>557</v>
       </c>
-      <c r="D3" s="24" t="s">
+      <c r="E3" s="26"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="25"/>
+      <c r="B4" s="25" t="s">
+        <v>553</v>
+      </c>
+      <c r="C4" s="24" t="s">
         <v>558</v>
       </c>
-      <c r="E3" s="25"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="24"/>
-      <c r="B4" s="24" t="s">
-        <v>554</v>
-      </c>
-      <c r="C4" s="23" t="s">
+      <c r="D4" s="25" t="s">
         <v>559</v>
       </c>
-      <c r="D4" s="24" t="s">
+      <c r="E4" s="26"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="25"/>
+      <c r="B5" s="25" t="s">
+        <v>553</v>
+      </c>
+      <c r="C5" s="24" t="s">
         <v>560</v>
       </c>
-      <c r="E4" s="25"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="24"/>
-      <c r="B5" s="24" t="s">
-        <v>554</v>
-      </c>
-      <c r="C5" s="23" t="s">
+      <c r="D5" s="25" t="s">
         <v>561</v>
       </c>
-      <c r="D5" s="24" t="s">
+      <c r="E5" s="26"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="25"/>
+      <c r="B6" s="25" t="s">
+        <v>553</v>
+      </c>
+      <c r="C6" s="24" t="s">
         <v>562</v>
       </c>
-      <c r="E5" s="25"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="24"/>
-      <c r="B6" s="24" t="s">
-        <v>554</v>
-      </c>
-      <c r="C6" s="23" t="s">
+      <c r="D6" s="25" t="s">
         <v>563</v>
       </c>
-      <c r="D6" s="24" t="s">
+      <c r="E6" s="26"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="25"/>
+      <c r="B7" s="25" t="s">
+        <v>553</v>
+      </c>
+      <c r="C7" s="24" t="s">
         <v>564</v>
       </c>
-      <c r="E6" s="25"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="24"/>
-      <c r="B7" s="24" t="s">
-        <v>554</v>
-      </c>
-      <c r="C7" s="23" t="s">
+      <c r="D7" s="25" t="s">
         <v>565</v>
       </c>
-      <c r="D7" s="24" t="s">
+      <c r="E7" s="26"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="27"/>
+      <c r="B8" s="28" t="s">
+        <v>553</v>
+      </c>
+      <c r="C8" s="29" t="s">
+        <v>480</v>
+      </c>
+      <c r="D8" s="28" t="s">
+        <v>481</v>
+      </c>
+      <c r="E8" s="26"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="27"/>
+      <c r="B9" s="28" t="s">
+        <v>553</v>
+      </c>
+      <c r="C9" s="29" t="s">
         <v>566</v>
       </c>
-      <c r="E7" s="25"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="26"/>
-      <c r="B8" s="27" t="s">
-        <v>554</v>
-      </c>
-      <c r="C8" s="28" t="s">
-        <v>481</v>
-      </c>
-      <c r="D8" s="27" t="s">
-        <v>482</v>
-      </c>
-      <c r="E8" s="25"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="26"/>
-      <c r="B9" s="27" t="s">
-        <v>554</v>
-      </c>
-      <c r="C9" s="28" t="s">
+      <c r="D9" s="28" t="s">
         <v>567</v>
       </c>
-      <c r="D9" s="27" t="s">
+      <c r="E9" s="26"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="27"/>
+      <c r="B10" s="28" t="s">
+        <v>553</v>
+      </c>
+      <c r="C10" s="29" t="s">
         <v>568</v>
       </c>
-      <c r="E9" s="25"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="26"/>
-      <c r="B10" s="27" t="s">
-        <v>554</v>
-      </c>
-      <c r="C10" s="28" t="s">
+      <c r="D10" s="28" t="s">
         <v>569</v>
       </c>
-      <c r="D10" s="27" t="s">
+      <c r="E10" s="26"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="27"/>
+      <c r="B11" s="28" t="s">
+        <v>553</v>
+      </c>
+      <c r="C11" s="29" t="s">
         <v>570</v>
       </c>
-      <c r="E10" s="25"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="26"/>
-      <c r="B11" s="27" t="s">
-        <v>554</v>
-      </c>
-      <c r="C11" s="29" t="s">
+      <c r="D11" s="28" t="s">
         <v>571</v>
       </c>
-      <c r="D11" s="30" t="s">
-        <v>572</v>
-      </c>
-      <c r="E11" s="25"/>
+      <c r="E11" s="26"/>
     </row>
     <row r="12">
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
@@ -9724,503 +9713,503 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="21" t="s">
+      <c r="B1" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="21" t="s">
+      <c r="C1" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="21" t="s">
+      <c r="D1" s="22" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="32" t="s">
+      <c r="E1" s="31" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="33" t="s">
+      <c r="A2" s="32" t="s">
+        <v>572</v>
+      </c>
+      <c r="B2" s="33" t="s">
         <v>573</v>
       </c>
-      <c r="B2" s="34" t="s">
+      <c r="C2" s="34" t="s">
         <v>574</v>
       </c>
-      <c r="C2" s="35" t="s">
+      <c r="D2" s="33" t="s">
         <v>575</v>
       </c>
-      <c r="D2" s="34" t="s">
+      <c r="E2" s="35" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="32" t="s">
         <v>576</v>
       </c>
-      <c r="E2" s="36" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="33" t="s">
+      <c r="B3" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="C3" s="34" t="s">
         <v>577</v>
       </c>
-      <c r="B3" s="34" t="s">
-        <v>574</v>
-      </c>
-      <c r="C3" s="35" t="s">
+      <c r="D3" s="33" t="s">
         <v>578</v>
       </c>
-      <c r="D3" s="34" t="s">
+      <c r="E3" s="35" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="32" t="s">
         <v>579</v>
       </c>
-      <c r="E3" s="36" t="s">
-        <v>563</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="33" t="s">
+      <c r="B4" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="C4" s="34" t="s">
         <v>580</v>
       </c>
-      <c r="B4" s="34" t="s">
-        <v>574</v>
-      </c>
-      <c r="C4" s="35" t="s">
+      <c r="D4" s="33" t="s">
         <v>581</v>
       </c>
-      <c r="D4" s="34" t="s">
+      <c r="E4" s="35" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="32" t="s">
         <v>582</v>
       </c>
-      <c r="E4" s="36" t="s">
-        <v>563</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="33" t="s">
+      <c r="B5" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="C5" s="34" t="s">
         <v>583</v>
       </c>
-      <c r="B5" s="34" t="s">
-        <v>574</v>
-      </c>
-      <c r="C5" s="35" t="s">
+      <c r="D5" s="33" t="s">
         <v>584</v>
       </c>
-      <c r="D5" s="34" t="s">
+      <c r="E5" s="35" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="32" t="s">
         <v>585</v>
       </c>
-      <c r="E5" s="36" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="33" t="s">
+      <c r="B6" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="C6" s="34" t="s">
         <v>586</v>
       </c>
-      <c r="B6" s="34" t="s">
-        <v>574</v>
-      </c>
-      <c r="C6" s="35" t="s">
+      <c r="D6" s="33" t="s">
         <v>587</v>
       </c>
-      <c r="D6" s="34" t="s">
+      <c r="E6" s="35" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="33"/>
+      <c r="B7" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="C7" s="34" t="s">
         <v>588</v>
       </c>
-      <c r="E6" s="36" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="34"/>
-      <c r="B7" s="34" t="s">
-        <v>574</v>
-      </c>
-      <c r="C7" s="35" t="s">
+      <c r="D7" s="33" t="s">
         <v>589</v>
       </c>
-      <c r="D7" s="34" t="s">
+      <c r="E7" s="35" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="33"/>
+      <c r="B8" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="C8" s="34" t="s">
         <v>590</v>
       </c>
-      <c r="E7" s="36" t="s">
-        <v>557</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="34"/>
-      <c r="B8" s="34" t="s">
-        <v>574</v>
-      </c>
-      <c r="C8" s="35" t="s">
+      <c r="D8" s="33" t="s">
         <v>591</v>
       </c>
-      <c r="D8" s="34" t="s">
+      <c r="E8" s="35" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="33"/>
+      <c r="B9" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="C9" s="34" t="s">
         <v>592</v>
       </c>
-      <c r="E8" s="36" t="s">
-        <v>555</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="34"/>
-      <c r="B9" s="34" t="s">
-        <v>574</v>
-      </c>
-      <c r="C9" s="35" t="s">
+      <c r="D9" s="33" t="s">
         <v>593</v>
       </c>
-      <c r="D9" s="34" t="s">
+      <c r="E9" s="35" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="33"/>
+      <c r="B10" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="C10" s="34" t="s">
         <v>594</v>
       </c>
-      <c r="E9" s="36" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="34"/>
-      <c r="B10" s="34" t="s">
-        <v>574</v>
-      </c>
-      <c r="C10" s="35" t="s">
+      <c r="D10" s="33" t="s">
         <v>595</v>
       </c>
-      <c r="D10" s="34" t="s">
+      <c r="E10" s="35" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="33"/>
+      <c r="B11" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="C11" s="34" t="s">
         <v>596</v>
       </c>
-      <c r="E10" s="36" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="34"/>
-      <c r="B11" s="34" t="s">
-        <v>574</v>
-      </c>
-      <c r="C11" s="35" t="s">
+      <c r="D11" s="33" t="s">
         <v>597</v>
       </c>
-      <c r="D11" s="34" t="s">
+      <c r="E11" s="35" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="33"/>
+      <c r="B12" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="C12" s="34" t="s">
         <v>598</v>
       </c>
-      <c r="E11" s="36" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="34"/>
-      <c r="B12" s="34" t="s">
-        <v>574</v>
-      </c>
-      <c r="C12" s="35" t="s">
+      <c r="D12" s="33" t="s">
         <v>599</v>
       </c>
-      <c r="D12" s="34" t="s">
+      <c r="E12" s="35" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="33"/>
+      <c r="B13" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="C13" s="34" t="s">
         <v>600</v>
       </c>
-      <c r="E12" s="36" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="34"/>
-      <c r="B13" s="34" t="s">
-        <v>574</v>
-      </c>
-      <c r="C13" s="35" t="s">
+      <c r="D13" s="33" t="s">
         <v>601</v>
       </c>
-      <c r="D13" s="34" t="s">
+      <c r="E13" s="35" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="33"/>
+      <c r="B14" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="C14" s="34" t="s">
         <v>602</v>
       </c>
-      <c r="E13" s="36" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="34"/>
-      <c r="B14" s="34" t="s">
-        <v>574</v>
-      </c>
-      <c r="C14" s="35" t="s">
+      <c r="D14" s="33" t="s">
         <v>603</v>
       </c>
-      <c r="D14" s="34" t="s">
+      <c r="E14" s="35" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="33"/>
+      <c r="B15" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="C15" s="34" t="s">
         <v>604</v>
       </c>
-      <c r="E14" s="36" t="s">
-        <v>563</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="34"/>
-      <c r="B15" s="34" t="s">
-        <v>574</v>
-      </c>
-      <c r="C15" s="35" t="s">
+      <c r="D15" s="33" t="s">
         <v>605</v>
       </c>
-      <c r="D15" s="34" t="s">
+      <c r="E15" s="35" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="33"/>
+      <c r="B16" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="C16" s="34" t="s">
         <v>606</v>
       </c>
-      <c r="E15" s="36" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="34"/>
-      <c r="B16" s="34" t="s">
-        <v>574</v>
-      </c>
-      <c r="C16" s="35" t="s">
+      <c r="D16" s="33" t="s">
         <v>607</v>
       </c>
-      <c r="D16" s="34" t="s">
+      <c r="E16" s="35" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="33"/>
+      <c r="B17" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="C17" s="34" t="s">
         <v>608</v>
       </c>
-      <c r="E16" s="36" t="s">
-        <v>563</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="34"/>
-      <c r="B17" s="34" t="s">
-        <v>574</v>
-      </c>
-      <c r="C17" s="35" t="s">
+      <c r="D17" s="33" t="s">
         <v>609</v>
       </c>
-      <c r="D17" s="34" t="s">
+      <c r="E17" s="35" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="33"/>
+      <c r="B18" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="C18" s="34" t="s">
         <v>610</v>
       </c>
-      <c r="E17" s="36" t="s">
-        <v>565</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="34"/>
-      <c r="B18" s="34" t="s">
-        <v>574</v>
-      </c>
-      <c r="C18" s="35" t="s">
+      <c r="D18" s="33" t="s">
         <v>611</v>
       </c>
-      <c r="D18" s="34" t="s">
+      <c r="E18" s="35" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="33"/>
+      <c r="B19" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="C19" s="34" t="s">
+        <v>570</v>
+      </c>
+      <c r="D19" s="33" t="s">
+        <v>571</v>
+      </c>
+      <c r="E19" s="35" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="33"/>
+      <c r="B20" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="C20" s="34" t="s">
         <v>612</v>
       </c>
-      <c r="E18" s="36" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="34"/>
-      <c r="B19" s="34" t="s">
-        <v>574</v>
-      </c>
-      <c r="C19" s="35" t="s">
-        <v>571</v>
-      </c>
-      <c r="D19" s="34" t="s">
-        <v>572</v>
-      </c>
-      <c r="E19" s="36" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="34"/>
-      <c r="B20" s="34" t="s">
-        <v>574</v>
-      </c>
-      <c r="C20" s="35" t="s">
+      <c r="D20" s="36" t="s">
         <v>613</v>
       </c>
-      <c r="D20" s="37" t="s">
+      <c r="E20" s="35" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="33"/>
+      <c r="B21" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="C21" s="34" t="s">
         <v>614</v>
       </c>
-      <c r="E20" s="36" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="34"/>
-      <c r="B21" s="34" t="s">
-        <v>574</v>
-      </c>
-      <c r="C21" s="35" t="s">
+      <c r="D21" s="33" t="s">
         <v>615</v>
       </c>
-      <c r="D21" s="34" t="s">
+      <c r="E21" s="35" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="33"/>
+      <c r="B22" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="C22" s="34" t="s">
         <v>616</v>
       </c>
-      <c r="E21" s="36" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="34"/>
-      <c r="B22" s="34" t="s">
-        <v>574</v>
-      </c>
-      <c r="C22" s="35" t="s">
+      <c r="D22" s="33" t="s">
         <v>617</v>
       </c>
-      <c r="D22" s="34" t="s">
+      <c r="E22" s="35" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="33"/>
+      <c r="B23" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="C23" s="34" t="s">
         <v>618</v>
       </c>
-      <c r="E22" s="36" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="34"/>
-      <c r="B23" s="34" t="s">
-        <v>574</v>
-      </c>
-      <c r="C23" s="35" t="s">
+      <c r="D23" s="33" t="s">
         <v>619</v>
       </c>
-      <c r="D23" s="34" t="s">
+      <c r="E23" s="35" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1">
+      <c r="A24" s="33"/>
+      <c r="B24" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="C24" s="34" t="s">
         <v>620</v>
       </c>
-      <c r="E23" s="36" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="34"/>
-      <c r="B24" s="34" t="s">
-        <v>574</v>
-      </c>
-      <c r="C24" s="35" t="s">
+      <c r="D24" s="33" t="s">
         <v>621</v>
       </c>
-      <c r="D24" s="34" t="s">
+      <c r="E24" s="35" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1">
+      <c r="A25" s="33"/>
+      <c r="B25" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="C25" s="34" t="s">
         <v>622</v>
       </c>
-      <c r="E24" s="36" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="34"/>
-      <c r="B25" s="34" t="s">
-        <v>574</v>
-      </c>
-      <c r="C25" s="35" t="s">
+      <c r="D25" s="33" t="s">
         <v>623</v>
       </c>
-      <c r="D25" s="34" t="s">
+      <c r="E25" s="35" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="26" ht="15.75" customHeight="1">
+      <c r="A26" s="33"/>
+      <c r="B26" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="C26" s="34" t="s">
         <v>624</v>
       </c>
-      <c r="E25" s="36" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="34"/>
-      <c r="B26" s="34" t="s">
-        <v>574</v>
-      </c>
-      <c r="C26" s="35" t="s">
+      <c r="D26" s="37" t="s">
         <v>625</v>
       </c>
-      <c r="D26" s="38" t="s">
+      <c r="E26" s="35" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="27" ht="15.75" customHeight="1">
+      <c r="A27" s="33"/>
+      <c r="B27" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="C27" s="34" t="s">
         <v>626</v>
       </c>
-      <c r="E26" s="36" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="34"/>
-      <c r="B27" s="34" t="s">
-        <v>574</v>
-      </c>
-      <c r="C27" s="35" t="s">
+      <c r="D27" s="33" t="s">
         <v>627</v>
       </c>
-      <c r="D27" s="34" t="s">
+      <c r="E27" s="35" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="28" ht="15.75" customHeight="1">
+      <c r="A28" s="33"/>
+      <c r="B28" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="C28" s="34" t="s">
         <v>628</v>
       </c>
-      <c r="E27" s="36" t="s">
-        <v>565</v>
-      </c>
-    </row>
-    <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="34"/>
-      <c r="B28" s="34" t="s">
-        <v>574</v>
-      </c>
-      <c r="C28" s="35" t="s">
+      <c r="D28" s="33" t="s">
         <v>629</v>
       </c>
-      <c r="D28" s="34" t="s">
+      <c r="E28" s="35" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="29" ht="15.75" customHeight="1">
+      <c r="A29" s="33"/>
+      <c r="B29" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="C29" s="34" t="s">
         <v>630</v>
       </c>
-      <c r="E28" s="36" t="s">
-        <v>559</v>
-      </c>
-    </row>
-    <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="34"/>
-      <c r="B29" s="34" t="s">
-        <v>574</v>
-      </c>
-      <c r="C29" s="35" t="s">
+      <c r="D29" s="33" t="s">
         <v>631</v>
       </c>
-      <c r="D29" s="34" t="s">
+      <c r="E29" s="35" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="30" ht="15.75" customHeight="1">
+      <c r="A30" s="33"/>
+      <c r="B30" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="C30" s="34" t="s">
+        <v>480</v>
+      </c>
+      <c r="D30" s="33" t="s">
+        <v>481</v>
+      </c>
+      <c r="E30" s="33"/>
+    </row>
+    <row r="31" ht="15.75" customHeight="1">
+      <c r="A31" s="33"/>
+      <c r="B31" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="C31" s="34" t="s">
+        <v>566</v>
+      </c>
+      <c r="D31" s="33" t="s">
         <v>632</v>
       </c>
-      <c r="E29" s="36" t="s">
-        <v>555</v>
-      </c>
-    </row>
-    <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="34"/>
-      <c r="B30" s="34" t="s">
-        <v>574</v>
-      </c>
-      <c r="C30" s="35" t="s">
-        <v>481</v>
-      </c>
-      <c r="D30" s="34" t="s">
-        <v>482</v>
-      </c>
-      <c r="E30" s="34"/>
-    </row>
-    <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="34"/>
-      <c r="B31" s="34" t="s">
-        <v>574</v>
-      </c>
-      <c r="C31" s="35" t="s">
-        <v>567</v>
-      </c>
-      <c r="D31" s="34" t="s">
+      <c r="E31" s="33"/>
+    </row>
+    <row r="32" ht="15.75" customHeight="1">
+      <c r="A32" s="33"/>
+      <c r="B32" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="C32" s="34" t="s">
+        <v>568</v>
+      </c>
+      <c r="D32" s="33" t="s">
         <v>633</v>
       </c>
-      <c r="E31" s="34"/>
-    </row>
-    <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="34"/>
-      <c r="B32" s="34" t="s">
-        <v>574</v>
-      </c>
-      <c r="C32" s="35" t="s">
-        <v>569</v>
-      </c>
-      <c r="D32" s="34" t="s">
+      <c r="E32" s="33"/>
+    </row>
+    <row r="33" ht="15.75" customHeight="1">
+      <c r="A33" s="33"/>
+      <c r="B33" s="33" t="s">
+        <v>573</v>
+      </c>
+      <c r="C33" s="34" t="s">
+        <v>560</v>
+      </c>
+      <c r="D33" s="33" t="s">
         <v>634</v>
       </c>
-      <c r="E32" s="34"/>
-    </row>
-    <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="34"/>
-      <c r="B33" s="34" t="s">
-        <v>574</v>
-      </c>
-      <c r="C33" s="35" t="s">
-        <v>561</v>
-      </c>
-      <c r="D33" s="34" t="s">
-        <v>635</v>
-      </c>
-      <c r="E33" s="34"/>
+      <c r="E33" s="33"/>
     </row>
     <row r="34" ht="15.75" customHeight="1"/>
     <row r="35" ht="15.75" customHeight="1"/>
@@ -11239,10 +11228,10 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
+        <v>635</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>636</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>637</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>95</v>
@@ -11254,22 +11243,22 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
+        <v>637</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>636</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>638</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>637</v>
-      </c>
-      <c r="C3" s="5" t="s">
+      <c r="D3" s="4" t="s">
         <v>639</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>640</v>
       </c>
       <c r="E3" s="4"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
@@ -12298,41 +12287,41 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
+        <v>641</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>642</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>643</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="D2" s="4" t="s">
         <v>644</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>645</v>
       </c>
       <c r="E2" s="4"/>
     </row>
     <row r="3">
       <c r="A3" s="4"/>
       <c r="B3" s="4" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="C3" s="5" t="s">
+        <v>645</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>646</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="E3" s="4"/>
+    </row>
+    <row r="4">
+      <c r="B4" s="13" t="s">
+        <v>642</v>
+      </c>
+      <c r="C4" s="12" t="s">
         <v>647</v>
       </c>
-      <c r="E3" s="4"/>
-    </row>
-    <row r="4">
-      <c r="B4" s="12" t="s">
-        <v>643</v>
-      </c>
-      <c r="C4" s="11" t="s">
+      <c r="D4" s="13" t="s">
         <v>648</v>
-      </c>
-      <c r="D4" s="12" t="s">
-        <v>649</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -13357,31 +13346,31 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
+        <v>649</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>650</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>651</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="D2" s="4" t="s">
         <v>652</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>653</v>
       </c>
       <c r="E2" s="4"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
+        <v>653</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>650</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>654</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>651</v>
-      </c>
-      <c r="C3" s="5" t="s">
+      <c r="D3" s="4" t="s">
         <v>655</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>656</v>
       </c>
       <c r="E3" s="4"/>
     </row>
@@ -14406,55 +14395,55 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="19" t="s">
+        <v>656</v>
+      </c>
+      <c r="B2" s="13" t="s">
         <v>657</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="C2" s="12" t="s">
         <v>658</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="D2" s="13" t="s">
         <v>659</v>
-      </c>
-      <c r="D2" s="12" t="s">
-        <v>660</v>
       </c>
       <c r="E2" s="4"/>
     </row>
     <row r="3">
       <c r="A3" s="4"/>
-      <c r="B3" s="12" t="s">
-        <v>658</v>
-      </c>
-      <c r="C3" s="11" t="s">
+      <c r="B3" s="13" t="s">
+        <v>657</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>660</v>
+      </c>
+      <c r="D3" s="13" t="s">
         <v>661</v>
-      </c>
-      <c r="D3" s="12" t="s">
-        <v>662</v>
       </c>
       <c r="E3" s="4"/>
     </row>
     <row r="4">
       <c r="A4" s="4"/>
-      <c r="B4" s="12" t="s">
-        <v>658</v>
-      </c>
-      <c r="C4" s="11" t="s">
+      <c r="B4" s="13" t="s">
+        <v>657</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>662</v>
+      </c>
+      <c r="D4" s="13" t="s">
         <v>663</v>
-      </c>
-      <c r="D4" s="12" t="s">
-        <v>664</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4"/>
-      <c r="B5" s="12" t="s">
-        <v>658</v>
-      </c>
-      <c r="C5" s="11" t="s">
+      <c r="B5" s="13" t="s">
+        <v>657</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>664</v>
+      </c>
+      <c r="D5" s="13" t="s">
         <v>665</v>
-      </c>
-      <c r="D5" s="12" t="s">
-        <v>666</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -21293,14 +21282,14 @@
       <c r="B3" s="4" t="s">
         <v>408</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>412</v>
+      <c r="C3" s="11" t="s">
+        <v>57</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>58</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="4">
@@ -21309,10 +21298,10 @@
         <v>408</v>
       </c>
       <c r="C4" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>414</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>415</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>327</v>
@@ -21324,13 +21313,13 @@
         <v>408</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>43</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="6">
@@ -21339,13 +21328,13 @@
         <v>408</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>76</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="7">
@@ -21360,7 +21349,7 @@
         <v>388</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="8">
@@ -21369,23 +21358,23 @@
         <v>408</v>
       </c>
       <c r="C8" s="5" t="s">
+        <v>420</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>421</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="E8" s="10" t="s">
         <v>422</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>423</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="4" t="s">
         <v>408</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="D9" s="12" t="s">
+      <c r="D9" s="13" t="s">
         <v>88</v>
       </c>
       <c r="E9" s="4"/>
@@ -22412,29 +22401,29 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
+        <v>423</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>424</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>425</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="D2" s="4" t="s">
         <v>426</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>427</v>
       </c>
       <c r="E2" s="4"/>
     </row>
     <row r="3">
       <c r="A3" s="4"/>
       <c r="B3" s="4" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="C3" s="5" t="s">
+        <v>427</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>428</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>429</v>
       </c>
       <c r="E3" s="4"/>
     </row>
@@ -23460,112 +23449,112 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
+        <v>429</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>430</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>431</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="D2" s="4" t="s">
         <v>432</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="E2" s="10" t="s">
         <v>433</v>
-      </c>
-      <c r="E2" s="10" t="s">
-        <v>434</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4"/>
       <c r="B3" s="4" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C3" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>435</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="E3" s="10" t="s">
         <v>436</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>437</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4"/>
       <c r="B4" s="4" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C4" s="5" t="s">
+        <v>437</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>438</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="E4" s="4" t="s">
         <v>439</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>440</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4"/>
       <c r="B5" s="4" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C5" s="5" t="s">
+        <v>440</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>441</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="E5" s="10" t="s">
         <v>442</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>443</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4"/>
       <c r="B6" s="4" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C6" s="5" t="s">
+        <v>443</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>444</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="E6" s="10" t="s">
         <v>445</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>446</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="4" t="s">
-        <v>431</v>
-      </c>
-      <c r="C7" s="13" t="s">
+        <v>430</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>446</v>
+      </c>
+      <c r="D7" s="15" t="s">
         <v>447</v>
-      </c>
-      <c r="D7" s="14" t="s">
-        <v>448</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="4" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C8" s="7" t="s">
+        <v>448</v>
+      </c>
+      <c r="D8" s="15" t="s">
         <v>449</v>
-      </c>
-      <c r="D8" s="14" t="s">
-        <v>450</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="4" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C9" s="7" t="s">
+        <v>450</v>
+      </c>
+      <c r="D9" s="15" t="s">
         <v>451</v>
-      </c>
-      <c r="D9" s="14" t="s">
-        <v>452</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -24590,25 +24579,25 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
+        <v>452</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>453</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>454</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="D2" s="4" t="s">
         <v>455</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="E2" s="10" t="s">
         <v>456</v>
-      </c>
-      <c r="E2" s="10" t="s">
-        <v>457</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4"/>
       <c r="B3" s="4" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>251</v>
@@ -24623,7 +24612,7 @@
     <row r="4">
       <c r="A4" s="4"/>
       <c r="B4" s="4" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>256</v>
@@ -24638,181 +24627,181 @@
     <row r="5">
       <c r="A5" s="4"/>
       <c r="B5" s="4" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="C5" s="5" t="s">
+        <v>457</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>458</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="E5" s="10" t="s">
         <v>459</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>460</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4"/>
       <c r="B6" s="4" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="C6" s="5" t="s">
+        <v>460</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>461</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="E6" s="10" t="s">
         <v>462</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>463</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4"/>
       <c r="B7" s="4" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="C7" s="5" t="s">
+        <v>463</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>464</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="E7" s="4" t="s">
         <v>465</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>466</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4"/>
       <c r="B8" s="4" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="C8" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>467</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="E8" s="10" t="s">
         <v>468</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>469</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4"/>
       <c r="B9" s="4" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="C9" s="5" t="s">
+        <v>469</v>
+      </c>
+      <c r="D9" s="4" t="s">
         <v>470</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="E9" s="10" t="s">
         <v>471</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>472</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4"/>
       <c r="B10" s="4" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>304</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4"/>
       <c r="B11" s="4" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="C11" s="5" t="s">
+        <v>474</v>
+      </c>
+      <c r="D11" s="4" t="s">
         <v>475</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="E11" s="10" t="s">
         <v>476</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>477</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4"/>
       <c r="B12" s="4" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="C12" s="5" t="s">
+        <v>477</v>
+      </c>
+      <c r="D12" s="4" t="s">
         <v>478</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="E12" s="10" t="s">
         <v>479</v>
-      </c>
-      <c r="E12" s="10" t="s">
-        <v>480</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4"/>
       <c r="B13" s="4" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="C13" s="5" t="s">
+        <v>480</v>
+      </c>
+      <c r="D13" s="4" t="s">
         <v>481</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="E13" s="10" t="s">
         <v>482</v>
-      </c>
-      <c r="E13" s="10" t="s">
-        <v>483</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4"/>
       <c r="B14" s="4" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>319</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4"/>
       <c r="B15" s="4" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="C15" s="5" t="s">
+        <v>485</v>
+      </c>
+      <c r="D15" s="4" t="s">
         <v>486</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="E15" s="10" t="s">
         <v>487</v>
-      </c>
-      <c r="E15" s="10" t="s">
-        <v>488</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4"/>
       <c r="B16" s="4" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="C16" s="5" t="s">
+        <v>488</v>
+      </c>
+      <c r="D16" s="4" t="s">
         <v>489</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="E16" s="4" t="s">
         <v>490</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>491</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>

</xml_diff>